<commit_message>
feat: perbarui logo daun tembakau dan posisikan pas di nota Excel dan web
</commit_message>
<xml_diff>
--- a/Nota/nota_142-147.xlsx
+++ b/Nota/nota_142-147.xlsx
@@ -208,6 +208,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="457200" cy="457200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -730,11 +760,11 @@
     <row r="17" ht="15.75" customHeight="1">
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>PPH 0,5%</t>
+          <t>PPH 1%</t>
         </is>
       </c>
       <c r="E17" s="12">
-        <f>CEILING(E16*0.005,5000)</f>
+        <f>CEILING(E16*0.01,5000)</f>
         <v/>
       </c>
     </row>
@@ -763,5 +793,6 @@
   </sheetData>
   <pageMargins left="1.062992125984252" right="0.1968503937007874" top="0.1968503937007874" bottom="0.1968503937007874" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>